<commit_message>
Add dashboard preview screenshot
</commit_message>
<xml_diff>
--- a/excel/renewable_energy_fpna_model.xlsx
+++ b/excel/renewable_energy_fpna_model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\renewable-energy-fpna-performance-model\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B4E18A-CF3C-48AE-A559-99D9E6326F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{968031F9-5B54-445F-9DEA-9227F6C909EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="601" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13180" tabRatio="601" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_ReadMe" sheetId="1" r:id="rId1"/>
@@ -1125,7 +1125,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1165,6 +1165,90 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1205,15 +1289,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1225,59 +1300,8 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1297,6 +1321,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1305,6 +1332,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1327,60 +1363,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1399,6 +1381,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1411,20 +1411,17 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -15677,8 +15674,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="299604" y="2570480"/>
-              <a:ext cx="8179724" cy="2743200"/>
+              <a:off x="300874" y="2586990"/>
+              <a:ext cx="8168294" cy="2762250"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -15877,8 +15874,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="0" y="6066626"/>
-              <a:ext cx="4235269" cy="4404408"/>
+              <a:off x="0" y="6103456"/>
+              <a:ext cx="4240349" cy="4432348"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -16501,124 +16498,124 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="43" t="s">
         <v>194</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="56"/>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="67" t="s">
         <v>195</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="69"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="72" t="s">
         <v>199</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="49"/>
-      <c r="K4" s="50"/>
+      <c r="B4" s="73"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="74"/>
+      <c r="J4" s="74"/>
+      <c r="K4" s="75"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="47"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="50"/>
+      <c r="A5" s="72"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="74"/>
+      <c r="K5" s="75"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="47"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="50"/>
+      <c r="A6" s="72"/>
+      <c r="B6" s="73"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="75"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="61"/>
-      <c r="B7" s="62"/>
-      <c r="C7" s="63"/>
-      <c r="D7" s="62"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
-      <c r="J7" s="63"/>
-      <c r="K7" s="64"/>
+      <c r="A7" s="55"/>
+      <c r="B7" s="56"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="56"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="58"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="70" t="s">
         <v>196</v>
       </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
+      <c r="B8" s="71"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="70"/>
+      <c r="H8" s="70"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="70"/>
+      <c r="K8" s="70"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="51" t="s">
+      <c r="A9" s="52" t="s">
         <v>200</v>
       </c>
-      <c r="B9" s="52"/>
+      <c r="B9" s="76"/>
       <c r="C9" s="53"/>
-      <c r="D9" s="52"/>
+      <c r="D9" s="76"/>
       <c r="E9" s="53"/>
       <c r="F9" s="53"/>
       <c r="G9" s="53"/>
@@ -16628,64 +16625,64 @@
       <c r="K9" s="54"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="44" t="s">
+      <c r="A10" s="49" t="s">
         <v>201</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="46"/>
+      <c r="B10" s="50"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="50"/>
+      <c r="G10" s="50"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="50"/>
+      <c r="K10" s="51"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="45"/>
-      <c r="K11" s="46"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="D11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="50"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="50"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="50"/>
+      <c r="K11" s="51"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="45"/>
-      <c r="K12" s="46"/>
+      <c r="B12" s="50"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="50"/>
+      <c r="G12" s="50"/>
+      <c r="H12" s="50"/>
+      <c r="I12" s="50"/>
+      <c r="J12" s="50"/>
+      <c r="K12" s="51"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="44" t="s">
+      <c r="A13" s="49" t="s">
         <v>204</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="45"/>
-      <c r="I13" s="45"/>
-      <c r="J13" s="45"/>
-      <c r="K13" s="46"/>
+      <c r="B13" s="50"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="50"/>
+      <c r="G13" s="50"/>
+      <c r="H13" s="50"/>
+      <c r="I13" s="50"/>
+      <c r="J13" s="50"/>
+      <c r="K13" s="51"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="8"/>
@@ -16701,22 +16698,22 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="66" t="s">
         <v>197</v>
       </c>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="38"/>
-      <c r="J15" s="38"/>
-      <c r="K15" s="38"/>
+      <c r="B15" s="66"/>
+      <c r="C15" s="66"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="66"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A16" s="51" t="s">
+      <c r="A16" s="52" t="s">
         <v>205</v>
       </c>
       <c r="B16" s="53"/>
@@ -16731,184 +16728,184 @@
       <c r="K16" s="54"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="49" t="s">
         <v>206</v>
       </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="45"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="45"/>
-      <c r="K17" s="46"/>
+      <c r="B17" s="50"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="50"/>
+      <c r="J17" s="50"/>
+      <c r="K17" s="51"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A18" s="44" t="s">
+      <c r="A18" s="49" t="s">
         <v>207</v>
       </c>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="46"/>
+      <c r="B18" s="50"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
+      <c r="J18" s="50"/>
+      <c r="K18" s="51"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A19" s="44" t="s">
+      <c r="A19" s="49" t="s">
         <v>208</v>
       </c>
-      <c r="B19" s="45"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="46"/>
+      <c r="B19" s="50"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A20" s="44" t="s">
+      <c r="A20" s="49" t="s">
         <v>209</v>
       </c>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="45"/>
-      <c r="K20" s="46"/>
+      <c r="B20" s="50"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="50"/>
+      <c r="G20" s="50"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="50"/>
+      <c r="K20" s="51"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A21" s="44" t="s">
+      <c r="A21" s="49" t="s">
         <v>210</v>
       </c>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="46"/>
+      <c r="B21" s="50"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="50"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="50"/>
+      <c r="K21" s="51"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="49" t="s">
         <v>211</v>
       </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="45"/>
-      <c r="K22" s="46"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
+      <c r="G22" s="50"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="50"/>
+      <c r="K22" s="51"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="49" t="s">
         <v>212</v>
       </c>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="46"/>
+      <c r="B23" s="50"/>
+      <c r="C23" s="50"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="50"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="50"/>
+      <c r="J23" s="50"/>
+      <c r="K23" s="51"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="49" t="s">
         <v>213</v>
       </c>
-      <c r="B24" s="45"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="45"/>
-      <c r="J24" s="45"/>
-      <c r="K24" s="46"/>
+      <c r="B24" s="50"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="50"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="50"/>
+      <c r="K24" s="51"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="49" t="s">
         <v>214</v>
       </c>
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="45"/>
-      <c r="J25" s="45"/>
-      <c r="K25" s="46"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="51"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="B26" s="57"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="58"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="45"/>
+      <c r="J26" s="45"/>
+      <c r="K26" s="46"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" s="57" t="s">
+      <c r="A27" s="45" t="s">
         <v>247</v>
       </c>
-      <c r="B27" s="57"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="58"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="45"/>
+      <c r="J27" s="45"/>
+      <c r="K27" s="46"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A28" s="59" t="s">
+      <c r="A28" s="47" t="s">
         <v>248</v>
       </c>
-      <c r="B28" s="59"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="59"/>
-      <c r="E28" s="59"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="59"/>
-      <c r="H28" s="59"/>
-      <c r="I28" s="59"/>
-      <c r="J28" s="59"/>
-      <c r="K28" s="60"/>
+      <c r="B28" s="47"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="48"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
@@ -16924,47 +16921,47 @@
       <c r="K29" s="7"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A30" s="31" t="s">
+      <c r="A30" s="59" t="s">
         <v>198</v>
       </c>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="31"/>
-      <c r="J30" s="31"/>
-      <c r="K30" s="31"/>
+      <c r="B30" s="59"/>
+      <c r="C30" s="59"/>
+      <c r="D30" s="59"/>
+      <c r="E30" s="59"/>
+      <c r="F30" s="59"/>
+      <c r="G30" s="59"/>
+      <c r="H30" s="59"/>
+      <c r="I30" s="59"/>
+      <c r="J30" s="59"/>
+      <c r="K30" s="59"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="60" t="s">
         <v>193</v>
       </c>
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="34"/>
+      <c r="B31" s="61"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
+      <c r="I31" s="61"/>
+      <c r="J31" s="61"/>
+      <c r="K31" s="62"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A32" s="35"/>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="36"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="36"/>
-      <c r="K32" s="37"/>
+      <c r="A32" s="63"/>
+      <c r="B32" s="64"/>
+      <c r="C32" s="64"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="64"/>
+      <c r="I32" s="64"/>
+      <c r="J32" s="64"/>
+      <c r="K32" s="65"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
@@ -16973,16 +16970,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:K2"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A27:K27"/>
-    <mergeCell ref="A28:K28"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A17:K17"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A10:K10"/>
-    <mergeCell ref="A7:K7"/>
     <mergeCell ref="A30:K30"/>
     <mergeCell ref="A31:K32"/>
     <mergeCell ref="A15:K15"/>
@@ -16999,6 +16986,16 @@
     <mergeCell ref="A13:K13"/>
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A1:K2"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A27:K27"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A18:K18"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A7:K7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17006,7 +17003,9 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{004C8D44-E1F4-4D63-9034-5560B3AD52A4}">
-  <sheetPr codeName="Sheet10"/>
+  <sheetPr codeName="Sheet10">
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -17020,74 +17019,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="B2" s="86"/>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
     </row>
     <row r="4" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="91"/>
-      <c r="D4" s="117" t="s">
+      <c r="B4" s="40"/>
+      <c r="D4" s="42" t="s">
         <v>124</v>
       </c>
-      <c r="E4" s="117"/>
-      <c r="G4" s="89" t="s">
+      <c r="E4" s="42"/>
+      <c r="G4" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="H4" s="89"/>
-      <c r="J4" s="89" t="s">
+      <c r="H4" s="38"/>
+      <c r="J4" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="K4" s="89"/>
+      <c r="K4" s="38"/>
     </row>
     <row r="5" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="92">
+      <c r="A5" s="41">
         <f>'06_Calculations'!B4</f>
         <v>136797930</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="D5" s="92">
+      <c r="B5" s="41"/>
+      <c r="D5" s="41">
         <f>'06_Calculations'!B7</f>
         <v>62995562</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="G5" s="92">
+      <c r="E5" s="41"/>
+      <c r="G5" s="41">
         <f>'06_Calculations'!E7</f>
         <v>-18246303</v>
       </c>
-      <c r="H5" s="92"/>
-      <c r="J5" s="90">
+      <c r="H5" s="41"/>
+      <c r="J5" s="39">
         <f>'06_Calculations'!E10</f>
         <v>947</v>
       </c>
-      <c r="K5" s="90"/>
+      <c r="K5" s="39"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B6" s="22"/>
@@ -17106,106 +17105,106 @@
       <c r="D9" s="22"/>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A58" s="87" t="s">
+      <c r="A58" s="36" t="s">
         <v>174</v>
       </c>
-      <c r="B58" s="87"/>
-      <c r="C58" s="87"/>
-      <c r="D58" s="87"/>
-      <c r="E58" s="87"/>
-      <c r="F58" s="87"/>
-      <c r="G58" s="87"/>
-      <c r="H58" s="87"/>
-      <c r="I58" s="87"/>
-      <c r="J58" s="87"/>
-      <c r="K58" s="87"/>
-      <c r="L58" s="87"/>
+      <c r="B58" s="36"/>
+      <c r="C58" s="36"/>
+      <c r="D58" s="36"/>
+      <c r="E58" s="36"/>
+      <c r="F58" s="36"/>
+      <c r="G58" s="36"/>
+      <c r="H58" s="36"/>
+      <c r="I58" s="36"/>
+      <c r="J58" s="36"/>
+      <c r="K58" s="36"/>
+      <c r="L58" s="36"/>
     </row>
     <row r="59" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="88" t="s">
+      <c r="A59" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="B59" s="88"/>
-      <c r="C59" s="88"/>
-      <c r="D59" s="88"/>
-      <c r="E59" s="88"/>
-      <c r="F59" s="88"/>
-      <c r="G59" s="88"/>
-      <c r="H59" s="88"/>
-      <c r="I59" s="88"/>
-      <c r="J59" s="88"/>
-      <c r="K59" s="88"/>
-      <c r="L59" s="88"/>
+      <c r="B59" s="37"/>
+      <c r="C59" s="37"/>
+      <c r="D59" s="37"/>
+      <c r="E59" s="37"/>
+      <c r="F59" s="37"/>
+      <c r="G59" s="37"/>
+      <c r="H59" s="37"/>
+      <c r="I59" s="37"/>
+      <c r="J59" s="37"/>
+      <c r="K59" s="37"/>
+      <c r="L59" s="37"/>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A60" s="88"/>
-      <c r="B60" s="88"/>
-      <c r="C60" s="88"/>
-      <c r="D60" s="88"/>
-      <c r="E60" s="88"/>
-      <c r="F60" s="88"/>
-      <c r="G60" s="88"/>
-      <c r="H60" s="88"/>
-      <c r="I60" s="88"/>
-      <c r="J60" s="88"/>
-      <c r="K60" s="88"/>
-      <c r="L60" s="88"/>
+      <c r="A60" s="37"/>
+      <c r="B60" s="37"/>
+      <c r="C60" s="37"/>
+      <c r="D60" s="37"/>
+      <c r="E60" s="37"/>
+      <c r="F60" s="37"/>
+      <c r="G60" s="37"/>
+      <c r="H60" s="37"/>
+      <c r="I60" s="37"/>
+      <c r="J60" s="37"/>
+      <c r="K60" s="37"/>
+      <c r="L60" s="37"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A61" s="88"/>
-      <c r="B61" s="88"/>
-      <c r="C61" s="88"/>
-      <c r="D61" s="88"/>
-      <c r="E61" s="88"/>
-      <c r="F61" s="88"/>
-      <c r="G61" s="88"/>
-      <c r="H61" s="88"/>
-      <c r="I61" s="88"/>
-      <c r="J61" s="88"/>
-      <c r="K61" s="88"/>
-      <c r="L61" s="88"/>
+      <c r="A61" s="37"/>
+      <c r="B61" s="37"/>
+      <c r="C61" s="37"/>
+      <c r="D61" s="37"/>
+      <c r="E61" s="37"/>
+      <c r="F61" s="37"/>
+      <c r="G61" s="37"/>
+      <c r="H61" s="37"/>
+      <c r="I61" s="37"/>
+      <c r="J61" s="37"/>
+      <c r="K61" s="37"/>
+      <c r="L61" s="37"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A62" s="88"/>
-      <c r="B62" s="88"/>
-      <c r="C62" s="88"/>
-      <c r="D62" s="88"/>
-      <c r="E62" s="88"/>
-      <c r="F62" s="88"/>
-      <c r="G62" s="88"/>
-      <c r="H62" s="88"/>
-      <c r="I62" s="88"/>
-      <c r="J62" s="88"/>
-      <c r="K62" s="88"/>
-      <c r="L62" s="88"/>
+      <c r="A62" s="37"/>
+      <c r="B62" s="37"/>
+      <c r="C62" s="37"/>
+      <c r="D62" s="37"/>
+      <c r="E62" s="37"/>
+      <c r="F62" s="37"/>
+      <c r="G62" s="37"/>
+      <c r="H62" s="37"/>
+      <c r="I62" s="37"/>
+      <c r="J62" s="37"/>
+      <c r="K62" s="37"/>
+      <c r="L62" s="37"/>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A63" s="88"/>
-      <c r="B63" s="88"/>
-      <c r="C63" s="88"/>
-      <c r="D63" s="88"/>
-      <c r="E63" s="88"/>
-      <c r="F63" s="88"/>
-      <c r="G63" s="88"/>
-      <c r="H63" s="88"/>
-      <c r="I63" s="88"/>
-      <c r="J63" s="88"/>
-      <c r="K63" s="88"/>
-      <c r="L63" s="88"/>
+      <c r="A63" s="37"/>
+      <c r="B63" s="37"/>
+      <c r="C63" s="37"/>
+      <c r="D63" s="37"/>
+      <c r="E63" s="37"/>
+      <c r="F63" s="37"/>
+      <c r="G63" s="37"/>
+      <c r="H63" s="37"/>
+      <c r="I63" s="37"/>
+      <c r="J63" s="37"/>
+      <c r="K63" s="37"/>
+      <c r="L63" s="37"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A64" s="88"/>
-      <c r="B64" s="88"/>
-      <c r="C64" s="88"/>
-      <c r="D64" s="88"/>
-      <c r="E64" s="88"/>
-      <c r="F64" s="88"/>
-      <c r="G64" s="88"/>
-      <c r="H64" s="88"/>
-      <c r="I64" s="88"/>
-      <c r="J64" s="88"/>
-      <c r="K64" s="88"/>
-      <c r="L64" s="88"/>
+      <c r="A64" s="37"/>
+      <c r="B64" s="37"/>
+      <c r="C64" s="37"/>
+      <c r="D64" s="37"/>
+      <c r="E64" s="37"/>
+      <c r="F64" s="37"/>
+      <c r="G64" s="37"/>
+      <c r="H64" s="37"/>
+      <c r="I64" s="37"/>
+      <c r="J64" s="37"/>
+      <c r="K64" s="37"/>
+      <c r="L64" s="37"/>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A65" s="4"/>
@@ -17268,8 +17267,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="7" scale="67" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -17280,218 +17280,218 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:19" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="97" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="104"/>
-      <c r="J1" s="104"/>
-      <c r="K1" s="104"/>
-      <c r="L1" s="104"/>
-      <c r="M1" s="104"/>
-      <c r="N1" s="104"/>
-      <c r="O1" s="104"/>
-      <c r="P1" s="104"/>
-      <c r="Q1" s="104"/>
-      <c r="R1" s="105"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="98"/>
+      <c r="Q1" s="98"/>
+      <c r="R1" s="99"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A2" s="106"/>
-      <c r="B2" s="107"/>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
-      <c r="Q2" s="107"/>
-      <c r="R2" s="108"/>
+      <c r="A2" s="100"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="101"/>
+      <c r="I2" s="101"/>
+      <c r="J2" s="101"/>
+      <c r="K2" s="101"/>
+      <c r="L2" s="101"/>
+      <c r="M2" s="101"/>
+      <c r="N2" s="101"/>
+      <c r="O2" s="101"/>
+      <c r="P2" s="101"/>
+      <c r="Q2" s="101"/>
+      <c r="R2" s="102"/>
     </row>
     <row r="3" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="106" t="s">
         <v>177</v>
       </c>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
-      <c r="L3" s="101"/>
-      <c r="M3" s="101"/>
-      <c r="N3" s="101"/>
-      <c r="O3" s="101"/>
-      <c r="P3" s="101"/>
-      <c r="Q3" s="101"/>
-      <c r="R3" s="102"/>
+      <c r="B3" s="107"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="107"/>
+      <c r="L3" s="107"/>
+      <c r="M3" s="107"/>
+      <c r="N3" s="107"/>
+      <c r="O3" s="107"/>
+      <c r="P3" s="107"/>
+      <c r="Q3" s="107"/>
+      <c r="R3" s="108"/>
     </row>
     <row r="4" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="96" t="s">
+      <c r="A4" s="103" t="s">
         <v>181</v>
       </c>
-      <c r="B4" s="115"/>
-      <c r="C4" s="115"/>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="99"/>
+      <c r="B4" s="104"/>
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="104"/>
+      <c r="M4" s="104"/>
+      <c r="N4" s="104"/>
+      <c r="O4" s="104"/>
+      <c r="P4" s="104"/>
+      <c r="Q4" s="104"/>
+      <c r="R4" s="105"/>
     </row>
     <row r="5" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="96"/>
-      <c r="B5" s="115"/>
-      <c r="C5" s="115"/>
-      <c r="D5" s="115"/>
-      <c r="E5" s="115"/>
-      <c r="F5" s="115"/>
-      <c r="G5" s="115"/>
-      <c r="H5" s="115"/>
-      <c r="I5" s="115"/>
-      <c r="J5" s="115"/>
-      <c r="K5" s="115"/>
-      <c r="L5" s="115"/>
-      <c r="M5" s="115"/>
-      <c r="N5" s="115"/>
-      <c r="O5" s="115"/>
-      <c r="P5" s="115"/>
-      <c r="Q5" s="115"/>
-      <c r="R5" s="99"/>
+      <c r="A5" s="103"/>
+      <c r="B5" s="104"/>
+      <c r="C5" s="104"/>
+      <c r="D5" s="104"/>
+      <c r="E5" s="104"/>
+      <c r="F5" s="104"/>
+      <c r="G5" s="104"/>
+      <c r="H5" s="104"/>
+      <c r="I5" s="104"/>
+      <c r="J5" s="104"/>
+      <c r="K5" s="104"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="104"/>
+      <c r="N5" s="104"/>
+      <c r="O5" s="104"/>
+      <c r="P5" s="104"/>
+      <c r="Q5" s="104"/>
+      <c r="R5" s="105"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A6" s="113"/>
-      <c r="B6" s="116"/>
-      <c r="C6" s="116"/>
-      <c r="D6" s="116"/>
-      <c r="E6" s="116"/>
-      <c r="F6" s="116"/>
-      <c r="G6" s="116"/>
-      <c r="H6" s="116"/>
-      <c r="I6" s="116"/>
-      <c r="J6" s="116"/>
-      <c r="K6" s="116"/>
-      <c r="L6" s="116"/>
-      <c r="M6" s="116"/>
-      <c r="N6" s="116"/>
-      <c r="O6" s="116"/>
-      <c r="P6" s="116"/>
-      <c r="Q6" s="116"/>
-      <c r="R6" s="114"/>
+      <c r="A6" s="31"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="33"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="32"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A7" s="100" t="s">
+      <c r="A7" s="106" t="s">
         <v>249</v>
       </c>
       <c r="B7" s="109"/>
-      <c r="C7" s="101"/>
+      <c r="C7" s="107"/>
       <c r="D7" s="109"/>
-      <c r="E7" s="101"/>
-      <c r="F7" s="101"/>
-      <c r="G7" s="101"/>
-      <c r="H7" s="101"/>
-      <c r="I7" s="101"/>
-      <c r="J7" s="101"/>
-      <c r="K7" s="101"/>
-      <c r="L7" s="101"/>
-      <c r="M7" s="101"/>
-      <c r="N7" s="101"/>
-      <c r="O7" s="101"/>
-      <c r="P7" s="101"/>
-      <c r="Q7" s="101"/>
-      <c r="R7" s="102"/>
+      <c r="E7" s="107"/>
+      <c r="F7" s="107"/>
+      <c r="G7" s="107"/>
+      <c r="H7" s="107"/>
+      <c r="I7" s="107"/>
+      <c r="J7" s="107"/>
+      <c r="K7" s="107"/>
+      <c r="L7" s="107"/>
+      <c r="M7" s="107"/>
+      <c r="N7" s="107"/>
+      <c r="O7" s="107"/>
+      <c r="P7" s="107"/>
+      <c r="Q7" s="107"/>
+      <c r="R7" s="108"/>
     </row>
     <row r="8" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="96" t="s">
+      <c r="A8" s="103" t="s">
         <v>182</v>
       </c>
-      <c r="B8" s="97"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="98"/>
-      <c r="H8" s="98"/>
-      <c r="I8" s="98"/>
-      <c r="J8" s="98"/>
-      <c r="K8" s="98"/>
-      <c r="L8" s="98"/>
-      <c r="M8" s="98"/>
-      <c r="N8" s="98"/>
-      <c r="O8" s="98"/>
-      <c r="P8" s="98"/>
-      <c r="Q8" s="98"/>
-      <c r="R8" s="99"/>
+      <c r="B8" s="116"/>
+      <c r="C8" s="104"/>
+      <c r="D8" s="116"/>
+      <c r="E8" s="104"/>
+      <c r="F8" s="104"/>
+      <c r="G8" s="104"/>
+      <c r="H8" s="104"/>
+      <c r="I8" s="104"/>
+      <c r="J8" s="104"/>
+      <c r="K8" s="104"/>
+      <c r="L8" s="104"/>
+      <c r="M8" s="104"/>
+      <c r="N8" s="104"/>
+      <c r="O8" s="104"/>
+      <c r="P8" s="104"/>
+      <c r="Q8" s="104"/>
+      <c r="R8" s="105"/>
     </row>
     <row r="9" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="96" t="s">
+      <c r="A9" s="103" t="s">
         <v>183</v>
       </c>
-      <c r="B9" s="97"/>
-      <c r="C9" s="98"/>
-      <c r="D9" s="97"/>
-      <c r="E9" s="98"/>
-      <c r="F9" s="98"/>
-      <c r="G9" s="98"/>
-      <c r="H9" s="98"/>
-      <c r="I9" s="98"/>
-      <c r="J9" s="98"/>
-      <c r="K9" s="98"/>
-      <c r="L9" s="98"/>
-      <c r="M9" s="98"/>
-      <c r="N9" s="98"/>
-      <c r="O9" s="98"/>
-      <c r="P9" s="98"/>
-      <c r="Q9" s="98"/>
-      <c r="R9" s="99"/>
+      <c r="B9" s="116"/>
+      <c r="C9" s="104"/>
+      <c r="D9" s="116"/>
+      <c r="E9" s="104"/>
+      <c r="F9" s="104"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="104"/>
+      <c r="I9" s="104"/>
+      <c r="J9" s="104"/>
+      <c r="K9" s="104"/>
+      <c r="L9" s="104"/>
+      <c r="M9" s="104"/>
+      <c r="N9" s="104"/>
+      <c r="O9" s="104"/>
+      <c r="P9" s="104"/>
+      <c r="Q9" s="104"/>
+      <c r="R9" s="105"/>
     </row>
     <row r="10" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="96" t="s">
+      <c r="A10" s="103" t="s">
         <v>184</v>
       </c>
-      <c r="B10" s="97"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="98"/>
-      <c r="H10" s="98"/>
-      <c r="I10" s="98"/>
-      <c r="J10" s="98"/>
-      <c r="K10" s="98"/>
-      <c r="L10" s="98"/>
-      <c r="M10" s="98"/>
-      <c r="N10" s="98"/>
-      <c r="O10" s="98"/>
-      <c r="P10" s="98"/>
-      <c r="Q10" s="98"/>
-      <c r="R10" s="99"/>
+      <c r="B10" s="116"/>
+      <c r="C10" s="104"/>
+      <c r="D10" s="116"/>
+      <c r="E10" s="104"/>
+      <c r="F10" s="104"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="104"/>
+      <c r="I10" s="104"/>
+      <c r="J10" s="104"/>
+      <c r="K10" s="104"/>
+      <c r="L10" s="104"/>
+      <c r="M10" s="104"/>
+      <c r="N10" s="104"/>
+      <c r="O10" s="104"/>
+      <c r="P10" s="104"/>
+      <c r="Q10" s="104"/>
+      <c r="R10" s="105"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
@@ -17537,92 +17537,92 @@
       <c r="S12" s="2"/>
     </row>
     <row r="13" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="96" t="s">
+      <c r="A13" s="103" t="s">
         <v>185</v>
       </c>
-      <c r="B13" s="98"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="98"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="98"/>
-      <c r="G13" s="98"/>
-      <c r="H13" s="98"/>
-      <c r="I13" s="98"/>
-      <c r="J13" s="98"/>
-      <c r="K13" s="98"/>
-      <c r="L13" s="98"/>
-      <c r="M13" s="98"/>
-      <c r="N13" s="98"/>
-      <c r="O13" s="98"/>
-      <c r="P13" s="98"/>
-      <c r="Q13" s="98"/>
-      <c r="R13" s="99"/>
+      <c r="B13" s="104"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="104"/>
+      <c r="E13" s="104"/>
+      <c r="F13" s="104"/>
+      <c r="G13" s="104"/>
+      <c r="H13" s="104"/>
+      <c r="I13" s="104"/>
+      <c r="J13" s="104"/>
+      <c r="K13" s="104"/>
+      <c r="L13" s="104"/>
+      <c r="M13" s="104"/>
+      <c r="N13" s="104"/>
+      <c r="O13" s="104"/>
+      <c r="P13" s="104"/>
+      <c r="Q13" s="104"/>
+      <c r="R13" s="105"/>
     </row>
     <row r="14" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="96" t="s">
+      <c r="A14" s="103" t="s">
         <v>186</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
-      <c r="H14" s="98"/>
-      <c r="I14" s="98"/>
-      <c r="J14" s="98"/>
-      <c r="K14" s="98"/>
-      <c r="L14" s="98"/>
-      <c r="M14" s="98"/>
-      <c r="N14" s="98"/>
-      <c r="O14" s="98"/>
-      <c r="P14" s="98"/>
-      <c r="Q14" s="98"/>
-      <c r="R14" s="99"/>
+      <c r="B14" s="104"/>
+      <c r="C14" s="104"/>
+      <c r="D14" s="104"/>
+      <c r="E14" s="104"/>
+      <c r="F14" s="104"/>
+      <c r="G14" s="104"/>
+      <c r="H14" s="104"/>
+      <c r="I14" s="104"/>
+      <c r="J14" s="104"/>
+      <c r="K14" s="104"/>
+      <c r="L14" s="104"/>
+      <c r="M14" s="104"/>
+      <c r="N14" s="104"/>
+      <c r="O14" s="104"/>
+      <c r="P14" s="104"/>
+      <c r="Q14" s="104"/>
+      <c r="R14" s="105"/>
     </row>
     <row r="15" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="96" t="s">
+      <c r="A15" s="103" t="s">
         <v>187</v>
       </c>
-      <c r="B15" s="98"/>
-      <c r="C15" s="98"/>
-      <c r="D15" s="98"/>
-      <c r="E15" s="98"/>
-      <c r="F15" s="98"/>
-      <c r="G15" s="98"/>
-      <c r="H15" s="98"/>
-      <c r="I15" s="98"/>
-      <c r="J15" s="98"/>
-      <c r="K15" s="98"/>
-      <c r="L15" s="98"/>
-      <c r="M15" s="98"/>
-      <c r="N15" s="98"/>
-      <c r="O15" s="98"/>
-      <c r="P15" s="98"/>
-      <c r="Q15" s="98"/>
-      <c r="R15" s="99"/>
+      <c r="B15" s="104"/>
+      <c r="C15" s="104"/>
+      <c r="D15" s="104"/>
+      <c r="E15" s="104"/>
+      <c r="F15" s="104"/>
+      <c r="G15" s="104"/>
+      <c r="H15" s="104"/>
+      <c r="I15" s="104"/>
+      <c r="J15" s="104"/>
+      <c r="K15" s="104"/>
+      <c r="L15" s="104"/>
+      <c r="M15" s="104"/>
+      <c r="N15" s="104"/>
+      <c r="O15" s="104"/>
+      <c r="P15" s="104"/>
+      <c r="Q15" s="104"/>
+      <c r="R15" s="105"/>
     </row>
     <row r="16" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="96" t="s">
+      <c r="A16" s="103" t="s">
         <v>188</v>
       </c>
-      <c r="B16" s="98"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="98"/>
-      <c r="E16" s="98"/>
-      <c r="F16" s="98"/>
-      <c r="G16" s="98"/>
-      <c r="H16" s="98"/>
-      <c r="I16" s="98"/>
-      <c r="J16" s="98"/>
-      <c r="K16" s="98"/>
-      <c r="L16" s="98"/>
-      <c r="M16" s="98"/>
-      <c r="N16" s="98"/>
-      <c r="O16" s="98"/>
-      <c r="P16" s="98"/>
-      <c r="Q16" s="98"/>
-      <c r="R16" s="99"/>
+      <c r="B16" s="104"/>
+      <c r="C16" s="104"/>
+      <c r="D16" s="104"/>
+      <c r="E16" s="104"/>
+      <c r="F16" s="104"/>
+      <c r="G16" s="104"/>
+      <c r="H16" s="104"/>
+      <c r="I16" s="104"/>
+      <c r="J16" s="104"/>
+      <c r="K16" s="104"/>
+      <c r="L16" s="104"/>
+      <c r="M16" s="104"/>
+      <c r="N16" s="104"/>
+      <c r="O16" s="104"/>
+      <c r="P16" s="104"/>
+      <c r="Q16" s="104"/>
+      <c r="R16" s="105"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
@@ -17645,114 +17645,114 @@
       <c r="R17" s="7"/>
     </row>
     <row r="18" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="100" t="s">
+      <c r="A18" s="106" t="s">
         <v>179</v>
       </c>
-      <c r="B18" s="101"/>
-      <c r="C18" s="101"/>
-      <c r="D18" s="101"/>
-      <c r="E18" s="101"/>
-      <c r="F18" s="101"/>
-      <c r="G18" s="101"/>
-      <c r="H18" s="101"/>
-      <c r="I18" s="101"/>
-      <c r="J18" s="101"/>
-      <c r="K18" s="101"/>
-      <c r="L18" s="101"/>
-      <c r="M18" s="101"/>
-      <c r="N18" s="101"/>
-      <c r="O18" s="101"/>
-      <c r="P18" s="101"/>
-      <c r="Q18" s="101"/>
-      <c r="R18" s="102"/>
+      <c r="B18" s="107"/>
+      <c r="C18" s="107"/>
+      <c r="D18" s="107"/>
+      <c r="E18" s="107"/>
+      <c r="F18" s="107"/>
+      <c r="G18" s="107"/>
+      <c r="H18" s="107"/>
+      <c r="I18" s="107"/>
+      <c r="J18" s="107"/>
+      <c r="K18" s="107"/>
+      <c r="L18" s="107"/>
+      <c r="M18" s="107"/>
+      <c r="N18" s="107"/>
+      <c r="O18" s="107"/>
+      <c r="P18" s="107"/>
+      <c r="Q18" s="107"/>
+      <c r="R18" s="108"/>
     </row>
     <row r="19" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="96" t="s">
+      <c r="A19" s="103" t="s">
         <v>189</v>
       </c>
-      <c r="B19" s="98"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="98"/>
-      <c r="E19" s="98"/>
-      <c r="F19" s="98"/>
-      <c r="G19" s="98"/>
-      <c r="H19" s="98"/>
-      <c r="I19" s="98"/>
-      <c r="J19" s="98"/>
-      <c r="K19" s="98"/>
-      <c r="L19" s="98"/>
-      <c r="M19" s="98"/>
-      <c r="N19" s="98"/>
-      <c r="O19" s="98"/>
-      <c r="P19" s="98"/>
-      <c r="Q19" s="98"/>
-      <c r="R19" s="99"/>
+      <c r="B19" s="104"/>
+      <c r="C19" s="104"/>
+      <c r="D19" s="104"/>
+      <c r="E19" s="104"/>
+      <c r="F19" s="104"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="104"/>
+      <c r="I19" s="104"/>
+      <c r="J19" s="104"/>
+      <c r="K19" s="104"/>
+      <c r="L19" s="104"/>
+      <c r="M19" s="104"/>
+      <c r="N19" s="104"/>
+      <c r="O19" s="104"/>
+      <c r="P19" s="104"/>
+      <c r="Q19" s="104"/>
+      <c r="R19" s="105"/>
     </row>
     <row r="20" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="96" t="s">
+      <c r="A20" s="103" t="s">
         <v>190</v>
       </c>
-      <c r="B20" s="98"/>
-      <c r="C20" s="98"/>
-      <c r="D20" s="98"/>
-      <c r="E20" s="98"/>
-      <c r="F20" s="98"/>
-      <c r="G20" s="98"/>
-      <c r="H20" s="98"/>
-      <c r="I20" s="98"/>
-      <c r="J20" s="98"/>
-      <c r="K20" s="98"/>
-      <c r="L20" s="98"/>
-      <c r="M20" s="98"/>
-      <c r="N20" s="98"/>
-      <c r="O20" s="98"/>
-      <c r="P20" s="98"/>
-      <c r="Q20" s="98"/>
-      <c r="R20" s="99"/>
+      <c r="B20" s="104"/>
+      <c r="C20" s="104"/>
+      <c r="D20" s="104"/>
+      <c r="E20" s="104"/>
+      <c r="F20" s="104"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="104"/>
+      <c r="I20" s="104"/>
+      <c r="J20" s="104"/>
+      <c r="K20" s="104"/>
+      <c r="L20" s="104"/>
+      <c r="M20" s="104"/>
+      <c r="N20" s="104"/>
+      <c r="O20" s="104"/>
+      <c r="P20" s="104"/>
+      <c r="Q20" s="104"/>
+      <c r="R20" s="105"/>
     </row>
     <row r="21" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="96" t="s">
+      <c r="A21" s="103" t="s">
         <v>191</v>
       </c>
-      <c r="B21" s="98"/>
-      <c r="C21" s="98"/>
-      <c r="D21" s="98"/>
-      <c r="E21" s="98"/>
-      <c r="F21" s="98"/>
-      <c r="G21" s="98"/>
-      <c r="H21" s="98"/>
-      <c r="I21" s="98"/>
-      <c r="J21" s="98"/>
-      <c r="K21" s="98"/>
-      <c r="L21" s="98"/>
-      <c r="M21" s="98"/>
-      <c r="N21" s="98"/>
-      <c r="O21" s="98"/>
-      <c r="P21" s="98"/>
-      <c r="Q21" s="98"/>
-      <c r="R21" s="99"/>
+      <c r="B21" s="104"/>
+      <c r="C21" s="104"/>
+      <c r="D21" s="104"/>
+      <c r="E21" s="104"/>
+      <c r="F21" s="104"/>
+      <c r="G21" s="104"/>
+      <c r="H21" s="104"/>
+      <c r="I21" s="104"/>
+      <c r="J21" s="104"/>
+      <c r="K21" s="104"/>
+      <c r="L21" s="104"/>
+      <c r="M21" s="104"/>
+      <c r="N21" s="104"/>
+      <c r="O21" s="104"/>
+      <c r="P21" s="104"/>
+      <c r="Q21" s="104"/>
+      <c r="R21" s="105"/>
     </row>
     <row r="22" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="96" t="s">
+      <c r="A22" s="103" t="s">
         <v>192</v>
       </c>
-      <c r="B22" s="98"/>
-      <c r="C22" s="98"/>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="F22" s="98"/>
-      <c r="G22" s="98"/>
-      <c r="H22" s="98"/>
-      <c r="I22" s="98"/>
-      <c r="J22" s="98"/>
-      <c r="K22" s="98"/>
-      <c r="L22" s="98"/>
-      <c r="M22" s="98"/>
-      <c r="N22" s="98"/>
-      <c r="O22" s="98"/>
-      <c r="P22" s="98"/>
-      <c r="Q22" s="98"/>
-      <c r="R22" s="99"/>
+      <c r="B22" s="104"/>
+      <c r="C22" s="104"/>
+      <c r="D22" s="104"/>
+      <c r="E22" s="104"/>
+      <c r="F22" s="104"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="104"/>
+      <c r="I22" s="104"/>
+      <c r="J22" s="104"/>
+      <c r="K22" s="104"/>
+      <c r="L22" s="104"/>
+      <c r="M22" s="104"/>
+      <c r="N22" s="104"/>
+      <c r="O22" s="104"/>
+      <c r="P22" s="104"/>
+      <c r="Q22" s="104"/>
+      <c r="R22" s="105"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
@@ -17771,64 +17771,55 @@
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
       <c r="P23" s="6"/>
-      <c r="Q23" s="63"/>
-      <c r="R23" s="64"/>
+      <c r="Q23" s="57"/>
+      <c r="R23" s="58"/>
     </row>
     <row r="24" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="93" t="s">
+      <c r="A24" s="113" t="s">
         <v>180</v>
       </c>
-      <c r="B24" s="94"/>
-      <c r="C24" s="94"/>
-      <c r="D24" s="94"/>
-      <c r="E24" s="94"/>
-      <c r="F24" s="94"/>
-      <c r="G24" s="94"/>
-      <c r="H24" s="94"/>
-      <c r="I24" s="94"/>
-      <c r="J24" s="94"/>
-      <c r="K24" s="94"/>
-      <c r="L24" s="94"/>
-      <c r="M24" s="94"/>
-      <c r="N24" s="94"/>
-      <c r="O24" s="94"/>
-      <c r="P24" s="94"/>
-      <c r="Q24" s="94"/>
-      <c r="R24" s="95"/>
+      <c r="B24" s="114"/>
+      <c r="C24" s="114"/>
+      <c r="D24" s="114"/>
+      <c r="E24" s="114"/>
+      <c r="F24" s="114"/>
+      <c r="G24" s="114"/>
+      <c r="H24" s="114"/>
+      <c r="I24" s="114"/>
+      <c r="J24" s="114"/>
+      <c r="K24" s="114"/>
+      <c r="L24" s="114"/>
+      <c r="M24" s="114"/>
+      <c r="N24" s="114"/>
+      <c r="O24" s="114"/>
+      <c r="P24" s="114"/>
+      <c r="Q24" s="114"/>
+      <c r="R24" s="115"/>
     </row>
     <row r="25" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="98" t="s">
+      <c r="A25" s="104" t="s">
         <v>193</v>
       </c>
-      <c r="B25" s="98"/>
-      <c r="C25" s="98"/>
-      <c r="D25" s="98"/>
-      <c r="E25" s="98"/>
-      <c r="F25" s="98"/>
-      <c r="G25" s="98"/>
-      <c r="H25" s="98"/>
-      <c r="I25" s="98"/>
-      <c r="J25" s="98"/>
-      <c r="K25" s="98"/>
-      <c r="L25" s="98"/>
-      <c r="M25" s="98"/>
-      <c r="N25" s="98"/>
-      <c r="O25" s="98"/>
-      <c r="P25" s="98"/>
-      <c r="Q25" s="98"/>
-      <c r="R25" s="98"/>
+      <c r="B25" s="104"/>
+      <c r="C25" s="104"/>
+      <c r="D25" s="104"/>
+      <c r="E25" s="104"/>
+      <c r="F25" s="104"/>
+      <c r="G25" s="104"/>
+      <c r="H25" s="104"/>
+      <c r="I25" s="104"/>
+      <c r="J25" s="104"/>
+      <c r="K25" s="104"/>
+      <c r="L25" s="104"/>
+      <c r="M25" s="104"/>
+      <c r="N25" s="104"/>
+      <c r="O25" s="104"/>
+      <c r="P25" s="104"/>
+      <c r="Q25" s="104"/>
+      <c r="R25" s="104"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A1:R2"/>
-    <mergeCell ref="A16:R16"/>
-    <mergeCell ref="A15:R15"/>
-    <mergeCell ref="A14:R14"/>
-    <mergeCell ref="A13:R13"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A7:R7"/>
-    <mergeCell ref="A12:R12"/>
-    <mergeCell ref="A4:R5"/>
     <mergeCell ref="A24:R24"/>
     <mergeCell ref="A8:R8"/>
     <mergeCell ref="A9:R9"/>
@@ -17840,6 +17831,15 @@
     <mergeCell ref="A20:R20"/>
     <mergeCell ref="A19:R19"/>
     <mergeCell ref="A18:R18"/>
+    <mergeCell ref="A1:R2"/>
+    <mergeCell ref="A16:R16"/>
+    <mergeCell ref="A15:R15"/>
+    <mergeCell ref="A14:R14"/>
+    <mergeCell ref="A13:R13"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A7:R7"/>
+    <mergeCell ref="A12:R12"/>
+    <mergeCell ref="A4:R5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -53087,447 +53087,455 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="77" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="71"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="79"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="72"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="74"/>
+      <c r="A2" s="80"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="81"/>
+      <c r="N2" s="82"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A3" s="65" t="s">
+      <c r="A3" s="87" t="s">
         <v>216</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="67"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="88"/>
+      <c r="K3" s="88"/>
+      <c r="L3" s="88"/>
+      <c r="M3" s="88"/>
+      <c r="N3" s="89"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="83" t="s">
         <v>220</v>
       </c>
-      <c r="B4" s="78"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="78"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="58"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
+      <c r="N4" s="46"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="83" t="s">
         <v>221</v>
       </c>
-      <c r="B5" s="78"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="78"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="58"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
+      <c r="N5" s="46"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" s="68" t="s">
+      <c r="A6" s="83" t="s">
         <v>222</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="78"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="57"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="58"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="45"/>
+      <c r="M6" s="45"/>
+      <c r="N6" s="46"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="68"/>
-      <c r="B7" s="78"/>
-      <c r="C7" s="57"/>
-      <c r="D7" s="78"/>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="57"/>
-      <c r="L7" s="57"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="58"/>
+      <c r="A7" s="83"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="90"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="45"/>
+      <c r="J7" s="45"/>
+      <c r="K7" s="45"/>
+      <c r="L7" s="45"/>
+      <c r="M7" s="45"/>
+      <c r="N7" s="46"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" s="65" t="s">
+      <c r="A8" s="87" t="s">
         <v>217</v>
       </c>
-      <c r="B8" s="79"/>
-      <c r="C8" s="66"/>
-      <c r="D8" s="79"/>
-      <c r="E8" s="66"/>
-      <c r="F8" s="66"/>
-      <c r="G8" s="66"/>
-      <c r="H8" s="66"/>
-      <c r="I8" s="66"/>
-      <c r="J8" s="66"/>
-      <c r="K8" s="66"/>
-      <c r="L8" s="66"/>
-      <c r="M8" s="66"/>
-      <c r="N8" s="67"/>
+      <c r="B8" s="91"/>
+      <c r="C8" s="88"/>
+      <c r="D8" s="91"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="88"/>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="89"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="83" t="s">
         <v>223</v>
       </c>
-      <c r="B9" s="78"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="78"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="57"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
-      <c r="N9" s="58"/>
+      <c r="B9" s="90"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="46"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="83" t="s">
         <v>224</v>
       </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="57"/>
-      <c r="J10" s="57"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="57"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="58"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="46"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A11" s="68" t="s">
+      <c r="A11" s="83" t="s">
         <v>225</v>
       </c>
-      <c r="B11" s="57"/>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
-      <c r="E11" s="57"/>
-      <c r="F11" s="57"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="57"/>
-      <c r="I11" s="57"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="57"/>
-      <c r="N11" s="58"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="46"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A12" s="68"/>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="57"/>
-      <c r="F12" s="57"/>
-      <c r="G12" s="57"/>
-      <c r="H12" s="57"/>
-      <c r="I12" s="57"/>
-      <c r="J12" s="57"/>
-      <c r="K12" s="57"/>
-      <c r="L12" s="57"/>
-      <c r="M12" s="57"/>
-      <c r="N12" s="58"/>
+      <c r="A12" s="83"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="45"/>
+      <c r="L12" s="45"/>
+      <c r="M12" s="45"/>
+      <c r="N12" s="46"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="68"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="57"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="57"/>
-      <c r="F13" s="57"/>
-      <c r="G13" s="57"/>
-      <c r="H13" s="57"/>
-      <c r="I13" s="57"/>
-      <c r="J13" s="57"/>
-      <c r="K13" s="57"/>
-      <c r="L13" s="57"/>
-      <c r="M13" s="57"/>
-      <c r="N13" s="58"/>
+      <c r="A13" s="83"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="45"/>
+      <c r="L13" s="45"/>
+      <c r="M13" s="45"/>
+      <c r="N13" s="46"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="87" t="s">
         <v>219</v>
       </c>
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="66"/>
-      <c r="L14" s="66"/>
-      <c r="M14" s="66"/>
-      <c r="N14" s="67"/>
+      <c r="B14" s="88"/>
+      <c r="C14" s="88"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="88"/>
+      <c r="F14" s="88"/>
+      <c r="G14" s="88"/>
+      <c r="H14" s="88"/>
+      <c r="I14" s="88"/>
+      <c r="J14" s="88"/>
+      <c r="K14" s="88"/>
+      <c r="L14" s="88"/>
+      <c r="M14" s="88"/>
+      <c r="N14" s="89"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A15" s="68" t="s">
+      <c r="A15" s="83" t="s">
         <v>226</v>
       </c>
-      <c r="B15" s="57"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="57"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="57"/>
-      <c r="L15" s="57"/>
-      <c r="M15" s="57"/>
-      <c r="N15" s="58"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="46"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A16" s="68" t="s">
+      <c r="A16" s="83" t="s">
         <v>227</v>
       </c>
-      <c r="B16" s="57"/>
-      <c r="C16" s="57"/>
-      <c r="D16" s="57"/>
-      <c r="E16" s="57"/>
-      <c r="F16" s="57"/>
-      <c r="G16" s="57"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
-      <c r="L16" s="57"/>
-      <c r="M16" s="57"/>
-      <c r="N16" s="58"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="45"/>
+      <c r="L16" s="45"/>
+      <c r="M16" s="45"/>
+      <c r="N16" s="46"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A17" s="68" t="s">
+      <c r="A17" s="83" t="s">
         <v>228</v>
       </c>
-      <c r="B17" s="57"/>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="57"/>
-      <c r="L17" s="57"/>
-      <c r="M17" s="57"/>
-      <c r="N17" s="58"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="46"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A18" s="68" t="s">
+      <c r="A18" s="83" t="s">
         <v>229</v>
       </c>
-      <c r="B18" s="57"/>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="57"/>
-      <c r="G18" s="57"/>
-      <c r="H18" s="57"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="57"/>
-      <c r="K18" s="57"/>
-      <c r="L18" s="57"/>
-      <c r="M18" s="57"/>
-      <c r="N18" s="58"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="45"/>
+      <c r="L18" s="45"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="46"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="83" t="s">
         <v>230</v>
       </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57"/>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57"/>
-      <c r="L19" s="57"/>
-      <c r="M19" s="57"/>
-      <c r="N19" s="58"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="45"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="45"/>
+      <c r="K19" s="45"/>
+      <c r="L19" s="45"/>
+      <c r="M19" s="45"/>
+      <c r="N19" s="46"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A20" s="68" t="s">
+      <c r="A20" s="83" t="s">
         <v>231</v>
       </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="57"/>
-      <c r="M20" s="57"/>
-      <c r="N20" s="58"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="45"/>
+      <c r="L20" s="45"/>
+      <c r="M20" s="45"/>
+      <c r="N20" s="46"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A21" s="61"/>
-      <c r="B21" s="63"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="63"/>
-      <c r="F21" s="63"/>
-      <c r="G21" s="63"/>
-      <c r="H21" s="63"/>
-      <c r="I21" s="63"/>
-      <c r="J21" s="63"/>
-      <c r="K21" s="63"/>
-      <c r="L21" s="63"/>
-      <c r="M21" s="63"/>
-      <c r="N21" s="64"/>
+      <c r="A21" s="55"/>
+      <c r="B21" s="57"/>
+      <c r="C21" s="57"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="57"/>
+      <c r="I21" s="57"/>
+      <c r="J21" s="57"/>
+      <c r="K21" s="57"/>
+      <c r="L21" s="57"/>
+      <c r="M21" s="57"/>
+      <c r="N21" s="58"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A22" s="65" t="s">
+      <c r="A22" s="87" t="s">
         <v>218</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="66"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="66"/>
-      <c r="I22" s="66"/>
-      <c r="J22" s="66"/>
-      <c r="K22" s="66"/>
-      <c r="L22" s="66"/>
-      <c r="M22" s="66"/>
-      <c r="N22" s="67"/>
+      <c r="B22" s="88"/>
+      <c r="C22" s="88"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="88"/>
+      <c r="G22" s="88"/>
+      <c r="H22" s="88"/>
+      <c r="I22" s="88"/>
+      <c r="J22" s="88"/>
+      <c r="K22" s="88"/>
+      <c r="L22" s="88"/>
+      <c r="M22" s="88"/>
+      <c r="N22" s="89"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A23" s="68" t="s">
+      <c r="A23" s="83" t="s">
         <v>232</v>
       </c>
-      <c r="B23" s="57"/>
-      <c r="C23" s="57"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="57"/>
-      <c r="L23" s="57"/>
-      <c r="M23" s="57"/>
-      <c r="N23" s="58"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="45"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="45"/>
+      <c r="L23" s="45"/>
+      <c r="M23" s="45"/>
+      <c r="N23" s="46"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A24" s="68" t="s">
+      <c r="A24" s="83" t="s">
         <v>233</v>
       </c>
-      <c r="B24" s="57"/>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="57"/>
-      <c r="K24" s="57"/>
-      <c r="L24" s="57"/>
-      <c r="M24" s="57"/>
-      <c r="N24" s="58"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="45"/>
+      <c r="K24" s="45"/>
+      <c r="L24" s="45"/>
+      <c r="M24" s="45"/>
+      <c r="N24" s="46"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A25" s="75" t="s">
+      <c r="A25" s="84" t="s">
         <v>234</v>
       </c>
-      <c r="B25" s="76"/>
-      <c r="C25" s="76"/>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="76"/>
-      <c r="I25" s="76"/>
-      <c r="J25" s="76"/>
-      <c r="K25" s="76"/>
-      <c r="L25" s="76"/>
-      <c r="M25" s="76"/>
-      <c r="N25" s="77"/>
+      <c r="B25" s="85"/>
+      <c r="C25" s="85"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="85"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="85"/>
+      <c r="I25" s="85"/>
+      <c r="J25" s="85"/>
+      <c r="K25" s="85"/>
+      <c r="L25" s="85"/>
+      <c r="M25" s="85"/>
+      <c r="N25" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A17:N17"/>
+    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A13:N13"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A11:N11"/>
+    <mergeCell ref="A10:N10"/>
     <mergeCell ref="A1:N2"/>
     <mergeCell ref="A16:N16"/>
     <mergeCell ref="A25:N25"/>
@@ -53544,14 +53552,6 @@
     <mergeCell ref="A6:N6"/>
     <mergeCell ref="A5:N5"/>
     <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A11:N11"/>
-    <mergeCell ref="A10:N10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -53568,18 +53568,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="92" t="s">
         <v>235</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="82"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="94"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="83"/>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="84"/>
+      <c r="A2" s="95"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="96"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">

</xml_diff>